<commit_message>
vault backup: 2026-07-22 18:02:11
</commit_message>
<xml_diff>
--- a/公司项目/认知行动/文档/软件需求跟踪矩阵.xlsx
+++ b/公司项目/认知行动/文档/软件需求跟踪矩阵.xlsx
@@ -2905,15 +2905,11 @@
       <x:c r="F34" s="3" t="str">
         <x:v>需求.md 舆情行动（目标识别与维护）</x:v>
       </x:c>
-      <x:c r="G34" s="3" t="inlineStr">
-        <x:is>
-          <x:t>M-OCC-01 目标档案与状态管理（目标数据管家）；M-OCC-03 目标关联网络（目标关系图谱）</x:t>
-        </x:is>
-      </x:c>
-      <x:c r="H34" s="3" t="inlineStr">
-        <x:is>
-          <x:t>F-OCC-01-01；F-OCC-01-02；F-OCC-01-03；F-OCC-01-04；F-OCC-01-05；F-OCC-03-01；F-OCC-03-02</x:t>
-        </x:is>
+      <x:c r="G34" s="3" t="str">
+        <x:v>M-OCC-01 目标档案与状态管理（目标数据管家）；M-OCC-02 目标关联网络（目标关系图谱）</x:v>
+      </x:c>
+      <x:c r="H34" s="3" t="str">
+        <x:v>F-OCC-01-01；F-OCC-01-02；F-OCC-01-03；F-OCC-01-04；F-OCC-01-05；F-OCC-02-01；F-OCC-02-02</x:v>
       </x:c>
       <x:c r="I34" s="3" t="inlineStr">
         <x:is>

</xml_diff>